<commit_message>
fix(data): pulihkan data entry anggaran 948 baris belanja ke dummy_data.xlsx
</commit_message>
<xml_diff>
--- a/data/template_upload.xlsx
+++ b/data/template_upload.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data Realisasi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Petunjuk Pengisian" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Data Realisasi Belanja" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data Realisasi Pendapatan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Petunjuk Pengisian" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,22 +41,22 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B3A5C"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <color rgb="001B3A5C"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00E74C3C"/>
+      <color rgb="000D5C3A"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +73,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D5C3A"/>
+        <bgColor rgb="000D5C3A"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,16 +122,16 @@
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,12 +506,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -663,356 +670,780 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>tahun</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>nama_opd</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>penanggungjawab</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kode_rekening</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kelompok_pendapatan</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>jenis_pendapatan</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>bulan</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>target_anggaran</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>realisasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Bidang Perbendaharaan</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>4.1.04.16.0001</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Pendapatan Asli Daerah (PAD)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Pendapatan Bunga Deposito Kas Daerah</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>18000000000</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>1200000000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Bidang Perbendaharaan</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>4.1.04.16.0002</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Pendapatan Asli Daerah (PAD)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Jasa Giro Rekening Kas Umum Daerah (RKUD)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>12500000000</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>950000000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Bidang Anggaran</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>4.2.01.02.0001</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Pendapatan Transfer</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Dana Alokasi Umum (DAU)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>620000000000</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>51666666667</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>PETUNJUK PENGISIAN TEMPLATE DATA REALISASI ANGGARAN BKAD</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>PETUNJUK PENGISIAN TEMPLATE DATA REALISASI ANGGARAN &amp; PENDAPATAN BKAD</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr"/>
+      <c r="A2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>A. PETUNJUK SHEET 'Data Realisasi Belanja'</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Kolom</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Tipe Data</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Contoh</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>tahun</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Angka (integer)</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Tahun anggaran (4 digit)</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>nama_opd</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Nama lengkap OPD</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>penanggungjawab</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Bidang penanggung jawab kegiatan</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Sekretariat / Bidang Anggaran / Bidang Perbendaharaan</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>kode_rekening</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Kode Rekening SIPD/SIMDA</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Kode Rekening Belanja SIPD (Akun 5.x)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>jenis_belanja</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Nama Sub-Kegiatan / Jenis Belanja</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>bulan</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Angka (1-12)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Bulan realisasi (1 = Jan, 12 = Des)</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>pagu_anggaran</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Angka (Rupiah)</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Pagu anggaran Rupiah penuh (tanpa titik/koma)</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>16342500</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>realisasi</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Angka (Rupiah)</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Nilai realisasi bulanan mentah Rupiah penuh pada bulan berkenaan</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>2440000</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>PENTING:</t>
-        </is>
-      </c>
+      <c r="A13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>1. Jangan mengubah nama kolom (baris pertama) pada sheet 'Data Realisasi'</t>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>B. PETUNJUK SHEET 'Data Realisasi Pendapatan'</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>2. Data realisasi diisi per bulan (mentah/non-kumulatif). Sistem Dashboard akan menghitung akumulasi secara otomatis</t>
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Kolom</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Tipe Data</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Contoh</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>3. Pagu anggaran bernilai SAMA untuk semua bulan dalam 1 tahun per kegiatan</t>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>tahun</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Angka (integer)</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Tahun anggaran (4 digit)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>4. Hapus 3 baris contoh (baris abu-abu) sebelum mengisi data asli</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>nama_opd</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Nama lengkap OPD</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>5. Simpan file dalam format .xlsx</t>
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>penanggungjawab</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Bidang penanggung jawab / pengelola pendapatan</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Bidang Perbendaharaan / Bidang Anggaran</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr"/>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>kode_rekening</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Kode Rekening Pendapatan SIPD (Akun 4.x)</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>4.1.04.16.0001</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>DAFTAR BIDANG PENANGGUNG JAWAB:</t>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>kelompok_pendapatan</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Kelompok: PAD / Pendapatan Transfer / Lain-lain Pendapatan Sah</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Pendapatan Asli Daerah (PAD)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>- Sekretariat</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>jenis_pendapatan</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Uraian nama akun pendapatan</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Pendapatan Bunga Deposito Kas Daerah</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>- Bidang Anggaran</t>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>bulan</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Angka (1-12)</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Bulan realisasi penerimaan (1 = Jan, 12 = Des)</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>- Bidang Perbendaharaan</t>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>target_anggaran</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Angka (Rupiah)</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Target pendapatan Rupiah penuh dalam 1 tahun</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>18000000000</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>- Bidang Akuntansi &amp; Pelaporan</t>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>realisasi</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Angka (Rupiah)</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Nilai realisasi penerimaan bulanan mentah pada bulan berkenaan</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>1200000000</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>- Bidang Pengelolaan BMD</t>
+      <c r="A25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>CATATAN PENTING:</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>1. Jangan mengubah nama kolom (baris pertama) pada sheet template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>2. Nilai realisasi diisi per bulan mentah (bukan kumulatif manual). Sistem akan menghitung akumulasi otomatis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>3. Pagu Belanja / Target Pendapatan bernilai sama untuk setiap bulan dalam tahun berkenaan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>4. Hapus baris contoh (warna abu-abu) sebelum mengunggah data resmi.</t>
         </is>
       </c>
     </row>

</xml_diff>